<commit_message>
add some new members and summer camp photo
</commit_message>
<xml_diff>
--- a/resources/membersalums_REF_ONLY.xlsx
+++ b/resources/membersalums_REF_ONLY.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\e-steam.github.io\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{214E4B0C-BEBD-427D-9D6A-FF886A76D234}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{723F0438-90A2-4042-855E-3AFC5AC19B0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{FDA1AC23-9684-4951-B0B2-FF55B1E34EAF}"/>
+    <workbookView xWindow="4485" yWindow="1005" windowWidth="22005" windowHeight="11295" xr2:uid="{FDA1AC23-9684-4951-B0B2-FF55B1E34EAF}"/>
   </bookViews>
   <sheets>
     <sheet name="Members" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="78">
   <si>
     <t>Name</t>
   </si>
@@ -244,6 +244,33 @@
   </si>
   <si>
     <t>Dr. Samantha Gilbert-Janizek</t>
+  </si>
+  <si>
+    <t>PhD Student in Earth and Space Sciences</t>
+  </si>
+  <si>
+    <t>resources/volunteers/ula_jones.jpg</t>
+  </si>
+  <si>
+    <t>Tiara Anderson</t>
+  </si>
+  <si>
+    <t>Ian Chow</t>
+  </si>
+  <si>
+    <t>Ella Marin</t>
+  </si>
+  <si>
+    <t>Dr. Joseph Murtagh</t>
+  </si>
+  <si>
+    <t>Angelina Zhang</t>
+  </si>
+  <si>
+    <t>resources/volunteers/tiara.jpg</t>
+  </si>
+  <si>
+    <t>resources/volunteers/ian_chow.jpg</t>
   </si>
 </sst>
 </file>
@@ -267,7 +294,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -286,6 +313,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -300,7 +333,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -308,6 +341,8 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -643,7 +678,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{30F2436D-6078-4782-A3F2-45402429735A}">
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.85546875" bestFit="1" customWidth="1"/>
@@ -716,91 +751,163 @@
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>26</v>
+      <c r="A6" s="5" t="s">
+        <v>35</v>
       </c>
       <c r="B6" t="s">
         <v>10</v>
       </c>
       <c r="C6" t="s">
-        <v>20</v>
-      </c>
-      <c r="E6" t="s">
-        <v>64</v>
+        <v>69</v>
+      </c>
+      <c r="D6" s="4"/>
+      <c r="E6" s="6" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B7" t="s">
-        <v>28</v>
+        <v>10</v>
       </c>
       <c r="C7" t="s">
         <v>20</v>
       </c>
-      <c r="D7" t="s">
-        <v>53</v>
-      </c>
       <c r="E7" t="s">
-        <v>54</v>
+        <v>64</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>51</v>
+        <v>27</v>
       </c>
       <c r="B8" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="C8" t="s">
         <v>20</v>
       </c>
+      <c r="D8" t="s">
+        <v>53</v>
+      </c>
       <c r="E8" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="B9" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="C9" t="s">
-        <v>56</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>67</v>
+        <v>20</v>
+      </c>
+      <c r="E9" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>36</v>
+        <v>55</v>
       </c>
       <c r="B10" t="s">
         <v>10</v>
       </c>
       <c r="C10" t="s">
+        <v>56</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>36</v>
+      </c>
+      <c r="B11" t="s">
+        <v>10</v>
+      </c>
+      <c r="C11" t="s">
         <v>65</v>
       </c>
-      <c r="E10" t="s">
+      <c r="E11" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="B12" s="2"/>
-      <c r="C12" s="2"/>
+      <c r="A12" t="s">
+        <v>71</v>
+      </c>
+      <c r="B12" t="s">
+        <v>10</v>
+      </c>
+      <c r="C12" t="s">
+        <v>20</v>
+      </c>
+      <c r="E12" t="s">
+        <v>76</v>
+      </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" s="2" t="s">
+      <c r="A13" t="s">
+        <v>72</v>
+      </c>
+      <c r="B13" t="s">
+        <v>15</v>
+      </c>
+      <c r="C13" t="s">
+        <v>20</v>
+      </c>
+      <c r="E13" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>73</v>
+      </c>
+      <c r="B14" s="2"/>
+      <c r="C14" s="2"/>
+      <c r="D14" s="2"/>
+      <c r="E14" s="2"/>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>74</v>
+      </c>
+      <c r="B15" s="2"/>
+      <c r="C15" s="2"/>
+      <c r="D15" s="2"/>
+      <c r="E15" s="2"/>
+    </row>
+    <row r="16" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>75</v>
+      </c>
+      <c r="B16" s="2"/>
+      <c r="C16" s="2"/>
+      <c r="D16" s="2"/>
+      <c r="E16" s="2"/>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" s="5"/>
+      <c r="B17" s="5"/>
+      <c r="C17" s="5"/>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="B13" s="2"/>
-      <c r="C13" s="2"/>
+      <c r="B18" s="5"/>
+      <c r="C18" s="5"/>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B19" s="5"/>
+      <c r="C19" s="5"/>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>

<commit_message>
add additional summer members
</commit_message>
<xml_diff>
--- a/resources/membersalums_REF_ONLY.xlsx
+++ b/resources/membersalums_REF_ONLY.xlsx
@@ -1,22 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\e-steam.github.io\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{723F0438-90A2-4042-855E-3AFC5AC19B0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CF15EFA-5E1B-4CC3-B68B-03BA50BCA485}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4485" yWindow="1005" windowWidth="22005" windowHeight="11295" xr2:uid="{FDA1AC23-9684-4951-B0B2-FF55B1E34EAF}"/>
+    <workbookView xWindow="4635" yWindow="3300" windowWidth="22005" windowHeight="11295" xr2:uid="{FDA1AC23-9684-4951-B0B2-FF55B1E34EAF}"/>
   </bookViews>
   <sheets>
     <sheet name="Members" sheetId="1" r:id="rId1"/>
     <sheet name="Alumni" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="84">
   <si>
     <t>Name</t>
   </si>
@@ -228,9 +229,6 @@
     <t>resources/volunteers/hurum.jpeg</t>
   </si>
   <si>
-    <t>Héctor Emanuel Delgado Díaz</t>
-  </si>
-  <si>
     <t>resources/volunteers/lainey.jpg</t>
   </si>
   <si>
@@ -271,6 +269,27 @@
   </si>
   <si>
     <t>resources/volunteers/ian_chow.jpg</t>
+  </si>
+  <si>
+    <t>resources/volunteers/joseph.png</t>
+  </si>
+  <si>
+    <t>resources/volunteers/ella.png</t>
+  </si>
+  <si>
+    <t>resources/volunteers/anna_grace.jpg</t>
+  </si>
+  <si>
+    <t>PhD Student in Earth and Space Sciences &amp; Astrobiology</t>
+  </si>
+  <si>
+    <t>Dr. Héctor Emanuel Delgado Díaz</t>
+  </si>
+  <si>
+    <t>PhD Student in Chemistry</t>
+  </si>
+  <si>
+    <t>resources/volunteers/angelina.png</t>
   </si>
 </sst>
 </file>
@@ -294,7 +313,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -313,12 +332,6 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC000"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -333,7 +346,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -342,7 +355,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -359,6 +371,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -678,12 +694,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{30F2436D-6078-4782-A3F2-45402429735A}">
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="37.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="51" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="36.7109375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="34.7109375" bestFit="1" customWidth="1"/>
   </cols>
@@ -721,93 +737,94 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>63</v>
+        <v>25</v>
       </c>
       <c r="B4" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="C4" t="s">
-        <v>17</v>
+        <v>20</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>61</v>
       </c>
       <c r="E4" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="B5" t="s">
         <v>10</v>
       </c>
       <c r="C5" t="s">
+        <v>68</v>
+      </c>
+      <c r="D5" s="4"/>
+      <c r="E5" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6" t="s">
         <v>20</v>
       </c>
-      <c r="D5" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="E5" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="B6" t="s">
-        <v>10</v>
-      </c>
-      <c r="C6" t="s">
-        <v>69</v>
-      </c>
-      <c r="D6" s="4"/>
-      <c r="E6" s="6" t="s">
-        <v>70</v>
+      <c r="E6" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B7" t="s">
-        <v>10</v>
+        <v>28</v>
       </c>
       <c r="C7" t="s">
         <v>20</v>
       </c>
+      <c r="D7" t="s">
+        <v>53</v>
+      </c>
       <c r="E7" t="s">
-        <v>64</v>
+        <v>54</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>27</v>
+        <v>51</v>
       </c>
       <c r="B8" t="s">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="C8" t="s">
         <v>20</v>
       </c>
-      <c r="D8" t="s">
-        <v>53</v>
-      </c>
       <c r="E8" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>51</v>
+        <v>34</v>
       </c>
       <c r="B9" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="C9" t="s">
-        <v>20</v>
-      </c>
+        <v>80</v>
+      </c>
+      <c r="D9" s="5"/>
       <c r="E9" t="s">
-        <v>52</v>
+        <v>79</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
@@ -821,7 +838,7 @@
         <v>56</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
@@ -832,15 +849,15 @@
         <v>10</v>
       </c>
       <c r="C11" t="s">
+        <v>64</v>
+      </c>
+      <c r="E11" t="s">
         <v>65</v>
-      </c>
-      <c r="E11" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B12" t="s">
         <v>10</v>
@@ -849,12 +866,12 @@
         <v>20</v>
       </c>
       <c r="E12" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B13" t="s">
         <v>15</v>
@@ -863,55 +880,57 @@
         <v>20</v>
       </c>
       <c r="E13" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>73</v>
-      </c>
-      <c r="B14" s="2"/>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
+        <v>72</v>
+      </c>
+      <c r="B14" t="s">
+        <v>10</v>
+      </c>
+      <c r="C14" t="s">
+        <v>20</v>
+      </c>
+      <c r="D14" s="5"/>
+      <c r="E14" t="s">
+        <v>78</v>
+      </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>74</v>
-      </c>
-      <c r="B15" s="2"/>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
+        <v>73</v>
+      </c>
+      <c r="B15" t="s">
+        <v>15</v>
+      </c>
+      <c r="C15" t="s">
+        <v>13</v>
+      </c>
+      <c r="D15" s="5"/>
+      <c r="E15" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="16" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>75</v>
-      </c>
-      <c r="B16" s="2"/>
-      <c r="C16" s="2"/>
-      <c r="D16" s="2"/>
-      <c r="E16" s="2"/>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" s="5"/>
-      <c r="B17" s="5"/>
-      <c r="C17" s="5"/>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="B18" s="5"/>
-      <c r="C18" s="5"/>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B19" s="5"/>
-      <c r="C19" s="5"/>
+        <v>74</v>
+      </c>
+      <c r="B16" t="s">
+        <v>10</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="D16" s="5"/>
+      <c r="E16" t="s">
+        <v>83</v>
+      </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="D5" r:id="rId1" display="http://htohfa.github.io/" xr:uid="{FF37C9DD-E8B0-48C0-8709-0F1F9DA2E8BD}"/>
+    <hyperlink ref="D4" r:id="rId1" display="http://htohfa.github.io/" xr:uid="{FF37C9DD-E8B0-48C0-8709-0F1F9DA2E8BD}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId2"/>
@@ -920,7 +939,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{22E1CA9D-58C7-4A5A-AD88-735485644128}">
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28" bestFit="1" customWidth="1"/>
@@ -1057,7 +1076,7 @@
       <c r="B9" t="s">
         <v>10</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="1" t="s">
         <v>50</v>
       </c>
       <c r="D9" t="s">
@@ -1103,7 +1122,7 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B12" t="s">
         <v>10</v>
@@ -1116,6 +1135,20 @@
       </c>
       <c r="E12" t="s">
         <v>38</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>81</v>
+      </c>
+      <c r="B13" t="s">
+        <v>15</v>
+      </c>
+      <c r="C13" t="s">
+        <v>17</v>
+      </c>
+      <c r="E13" t="s">
+        <v>60</v>
       </c>
     </row>
   </sheetData>

</xml_diff>